<commit_message>
Finish Data Automation Tool v1 with README and tests
</commit_message>
<xml_diff>
--- a/reports/sales_report.xlsx
+++ b/reports/sales_report.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,6 +453,11 @@
           <t>city</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>amount_in_eur</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -479,6 +484,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="G2" t="n">
+        <v>13.84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -505,6 +513,9 @@
           <t>Orlando</t>
         </is>
       </c>
+      <c r="G3" t="n">
+        <v>19.48</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -531,6 +542,9 @@
           <t>Tampa</t>
         </is>
       </c>
+      <c r="G4" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -557,6 +571,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>735.95</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -583,6 +600,9 @@
           <t>Orlando</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -609,6 +629,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="G7" t="n">
+        <v>129.87</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -634,6 +657,9 @@
         <is>
           <t>Jacksonville</t>
         </is>
+      </c>
+      <c r="G8" t="n">
+        <v>22.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>